<commit_message>
Add prototype character audio and effects
</commit_message>
<xml_diff>
--- a/asset_manifest.xlsx
+++ b/asset_manifest.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" r:id="Rf1c31449ce284d97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset - Trận địa cọc" sheetId="2" r:id="R1c04db1444a24e58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prefix" sheetId="3" r:id="Rcb07be42773f48cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hướng dẫn" sheetId="4" r:id="Ref2b02385d4b4084"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" r:id="R223ae6e09e854af5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset - Trận địa cọc" sheetId="2" r:id="Rd60bef940a1b4ae7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prefix" sheetId="3" r:id="R21c78b134bbe41b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hướng dẫn" sheetId="4" r:id="Rf988d09c8eb84f9b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -40,25 +40,13 @@
     <x:t xml:space="preserve">Trạng thái còn lại</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">8 hạng mục chưa có, để làm sau</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Lưu ý về reference</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Đã bỏ reference khỏi danh sách asset chính; file vẫn giữ trong thư mục REFERENCE.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">BGM và VO</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Nhạc sảnh, nhạc gameplay và battle call chưa có; để làm sau.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Quyền sử dụng</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Tệp tự tạo; nhạc và voice mới cần xác nhận quyền sử dụng.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Dữ liệu lịch sử</x:t>
@@ -683,15 +671,15 @@
       <x:c r="A6" s="6" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B6" s="2">
-        <x:v>43</x:v>
+      <x:c r="B6" s="2" t="n">
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B7" s="2">
+      <x:c r="B7" s="2" t="n">
         <x:v>6</x:v>
       </x:c>
     </x:row>
@@ -699,40 +687,40 @@
       <x:c r="A8" s="6" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B8" s="2" t="s">
-        <x:v>9</x:v>
+      <x:c r="B8" s="2" t="str">
+        <x:v>1 hạng mục chưa có, để làm sau</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="6" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B9" s="2" t="s">
-        <x:v>11</x:v>
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B9" s="2" t="str">
+        <x:v>Đã bỏ reference khỏi danh sách asset chính; file vẫn giữ trong thư mục REFERENCE.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="6" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B10" s="2" t="s">
-        <x:v>13</x:v>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B10" s="2" t="str">
+        <x:v>Đã bổ sung BGM prototype, trống prototype và script battle call; voice thật còn chờ thu/tạo có cấp phép.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="6" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B11" s="2" t="s">
-        <x:v>15</x:v>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B11" s="2" t="str">
+        <x:v>Asset tự tạo và font Be Vietnam Pro có OFL; voice cuối cần xác nhận quyền sử dụng.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="6" t="s">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B12" s="2" t="s">
-        <x:v>17</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -1309,17 +1297,19 @@
         <x:v>lobby_theme</x:v>
       </x:c>
       <x:c r="E17" s="2" t="str">
-        <x:v>Nhạc nền sảnh loop 60–90 giây</x:v>
+        <x:v>Nhạc nền sảnh prototype loop 16 giây, tự tạo; bản chính thức có thể remaster thành 60–90 giây</x:v>
       </x:c>
       <x:c r="F17" s="2" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G17" s="3" t="str">
-        <x:v>Chưa có (làm sau)</x:v>
-      </x:c>
-      <x:c r="H17" s="2"/>
+        <x:v>Đã có</x:v>
+      </x:c>
+      <x:c r="H17" s="2" t="str">
+        <x:v>https://github.com/mil352k5-ux/MiniGame_TranDiaCocBD/blob/main/BGM/lobby_theme_prototype.wav</x:v>
+      </x:c>
       <x:c r="I17" s="2" t="str">
-        <x:v>BGM/lobby_theme.mp3</x:v>
+        <x:v>BGM/lobby_theme_prototype.wav</x:v>
       </x:c>
       <x:c r="J17" s="2" t="str">
         <x:v>P1</x:v>
@@ -1439,16 +1429,20 @@
         <x:v>CHR_NgoQuyen_HighRes</x:v>
       </x:c>
       <x:c r="E21" s="2" t="str">
-        <x:v>Phiên bản nhân vật độ phân giải cao, đã tách 3 pose; chỉ sau duyệt concept</x:v>
+        <x:v>3 pose PNG độ phân giải cao, nền trong suốt; chờ duyệt concept trước bản chính thức</x:v>
       </x:c>
       <x:c r="F21" s="2" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G21" s="3" t="str">
-        <x:v>Chưa có (làm sau)</x:v>
-      </x:c>
-      <x:c r="H21" s="2"/>
-      <x:c r="I21" s="2"/>
+        <x:v>Đã có</x:v>
+      </x:c>
+      <x:c r="H21" s="2" t="str">
+        <x:v>https://github.com/mil352k5-ux/MiniGame_TranDiaCocBD/tree/main/CHR</x:v>
+      </x:c>
+      <x:c r="I21" s="2" t="str">
+        <x:v>CHR/ngo_quyen_highres_idle.png; CHR/ngo_quyen_highres_command.png; CHR/ngo_quyen_highres_victory.png</x:v>
+      </x:c>
       <x:c r="J21" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
@@ -1633,16 +1627,20 @@
         <x:v>ANM_CloakRig</x:v>
       </x:c>
       <x:c r="E27" s="2" t="str">
-        <x:v>Áo choàng lay động nhẹ theo gió; chưa dựng sprite rig</x:v>
+        <x:v>Lớp áo choàng SVG tùy chọn và hợp đồng tween</x:v>
       </x:c>
       <x:c r="F27" s="2" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G27" s="3" t="str">
-        <x:v>Chưa có (làm sau)</x:v>
-      </x:c>
-      <x:c r="H27" s="2"/>
-      <x:c r="I27" s="2"/>
+        <x:v>Đã có</x:v>
+      </x:c>
+      <x:c r="H27" s="2" t="str">
+        <x:v>https://github.com/mil352k5-ux/MiniGame_TranDiaCocBD/blob/main/ANM/cloak_rig_contract.json</x:v>
+      </x:c>
+      <x:c r="I27" s="2" t="str">
+        <x:v>ANM/cloak_rig_contract.json; CHR/ngo_quyen_cloak_back.svg; CHR/ngo_quyen_cloak_front.svg</x:v>
+      </x:c>
       <x:c r="J27" s="2" t="str">
         <x:v>P2</x:v>
       </x:c>
@@ -1662,17 +1660,19 @@
         <x:v>gameplay_theme</x:v>
       </x:c>
       <x:c r="E28" s="2" t="str">
-        <x:v>Nhạc nền gameplay loop 90–120 giây</x:v>
+        <x:v>Nhạc nền gameplay prototype loop 16 giây, tự tạo; bản chính thức có thể mở rộng 90–120 giây</x:v>
       </x:c>
       <x:c r="F28" s="2" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G28" s="3" t="str">
-        <x:v>Chưa có (làm sau)</x:v>
-      </x:c>
-      <x:c r="H28" s="2"/>
+        <x:v>Đã có</x:v>
+      </x:c>
+      <x:c r="H28" s="2" t="str">
+        <x:v>https://github.com/mil352k5-ux/MiniGame_TranDiaCocBD/blob/main/BGM/gameplay_theme_prototype.wav</x:v>
+      </x:c>
       <x:c r="I28" s="2" t="str">
-        <x:v>BGM/gameplay_theme.mp3</x:v>
+        <x:v>BGM/gameplay_theme_prototype.wav</x:v>
       </x:c>
       <x:c r="J28" s="2" t="str">
         <x:v>P1</x:v>
@@ -1858,16 +1858,20 @@
         <x:v>VFX_AdvancedFoam</x:v>
       </x:c>
       <x:c r="E34" s="2" t="str">
-        <x:v>Bọt sóng nâng cao, chưa hoàn thiện</x:v>
+        <x:v>Bọt sóng nâng cao dạng SVG cho phản công</x:v>
       </x:c>
       <x:c r="F34" s="2" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G34" s="3" t="str">
-        <x:v>Chưa có (làm sau)</x:v>
-      </x:c>
-      <x:c r="H34" s="2"/>
-      <x:c r="I34" s="2"/>
+        <x:v>Đã có</x:v>
+      </x:c>
+      <x:c r="H34" s="2" t="str">
+        <x:v>https://github.com/mil352k5-ux/MiniGame_TranDiaCocBD/blob/main/VFX/advanced_foam.svg</x:v>
+      </x:c>
+      <x:c r="I34" s="2" t="str">
+        <x:v>VFX/advanced_foam.svg</x:v>
+      </x:c>
       <x:c r="J34" s="2" t="str">
         <x:v>P2</x:v>
       </x:c>
@@ -2151,16 +2155,20 @@
         <x:v>SFX_VietnameseDrum</x:v>
       </x:c>
       <x:c r="E43" s="2" t="str">
-        <x:v>Nhạc cụ / trống phù hợp có quyền sử dụng hoặc tự thu âm</x:v>
+        <x:v>Một hit trống prototype tự tạo; cần thay/remaster nếu muốn chất liệu trống Việt Nam rõ hơn</x:v>
       </x:c>
       <x:c r="F43" s="2" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G43" s="5" t="str">
-        <x:v>Chưa có (làm sau)</x:v>
-      </x:c>
-      <x:c r="H43" s="2"/>
-      <x:c r="I43" s="2"/>
+        <x:v>Đã có</x:v>
+      </x:c>
+      <x:c r="H43" s="2" t="str">
+        <x:v>https://github.com/mil352k5-ux/MiniGame_TranDiaCocBD/blob/main/SFX/vietnamese_drum_prototype.wav</x:v>
+      </x:c>
+      <x:c r="I43" s="2" t="str">
+        <x:v>SFX/vietnamese_drum_prototype.wav</x:v>
+      </x:c>
       <x:c r="J43" s="2" t="str">
         <x:v>P2</x:v>
       </x:c>
@@ -2279,7 +2287,7 @@
         <x:v>battle_calls</x:v>
       </x:c>
       <x:c r="E47" s="2" t="str">
-        <x:v>Lời hô ngắn: Nước rút, Giữ trận địa, Thả cọc, Phản công</x:v>
+        <x:v>Kịch bản 5 câu đã chuẩn bị; cần thu hoặc tạo voice tiếng Việt có quyền sử dụng</x:v>
       </x:c>
       <x:c r="F47" s="2" t="str">
         <x:v>4–6 câu</x:v>
@@ -2287,9 +2295,11 @@
       <x:c r="G47" s="5" t="str">
         <x:v>Chưa có (làm sau)</x:v>
       </x:c>
-      <x:c r="H47" s="2"/>
+      <x:c r="H47" s="2" t="str">
+        <x:v>https://github.com/mil352k5-ux/MiniGame_TranDiaCocBD/blob/main/VO/battle_calls_script.json</x:v>
+      </x:c>
       <x:c r="I47" s="2" t="str">
-        <x:v>VO/battle_calls/</x:v>
+        <x:v>VO/battle_calls_script.json</x:v>
       </x:c>
       <x:c r="J47" s="2" t="str">
         <x:v>P1</x:v>
@@ -2409,16 +2419,20 @@
         <x:v>FONT_VietnameseLicensed</x:v>
       </x:c>
       <x:c r="E51" t="str">
-        <x:v>Font bản địa hỗ trợ đầy đủ dấu tiếng Việt và quyền phân phối rõ ràng; demo dùng fallback hệ thống</x:v>
+        <x:v>Be Vietnam Pro Regular/Bold, giấy phép SIL Open Font License 1.1</x:v>
       </x:c>
       <x:c r="F51" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G51" t="str">
-        <x:v>Chưa có (làm sau)</x:v>
-      </x:c>
-      <x:c r="H51"/>
-      <x:c r="I51"/>
+        <x:v>Đã có</x:v>
+      </x:c>
+      <x:c r="H51" t="str">
+        <x:v>https://github.com/mil352k5-ux/MiniGame_TranDiaCocBD/tree/main/FONT</x:v>
+      </x:c>
+      <x:c r="I51" t="str">
+        <x:v>FONT/BeVietnamPro-Regular.ttf; FONT/BeVietnamPro-Bold.ttf; FONT/OFL.txt</x:v>
+      </x:c>
       <x:c r="J51" t="str">
         <x:v>P1</x:v>
       </x:c>
@@ -2479,212 +2493,212 @@
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
       <x:c r="A1" s="7" t="s">
-        <x:v>18</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B1" s="7" t="s">
-        <x:v>19</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C1" s="7" t="s">
-        <x:v>20</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D1" s="7" t="s">
-        <x:v>21</x:v>
+        <x:v>17</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="s">
-        <x:v>22</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B2" t="s">
-        <x:v>23</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C2" t="s">
-        <x:v>24</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D2" t="s">
-        <x:v>25</x:v>
+        <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="s">
-        <x:v>26</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B3" t="s">
-        <x:v>27</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C3" t="s">
-        <x:v>28</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D3" t="s">
-        <x:v>29</x:v>
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="s">
-        <x:v>30</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B4" t="s">
-        <x:v>31</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="C4" t="s">
-        <x:v>32</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="D4" t="s">
-        <x:v>33</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="s">
-        <x:v>34</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B5" t="s">
-        <x:v>35</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="C5" t="s">
-        <x:v>36</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="D5" t="s">
-        <x:v>37</x:v>
+        <x:v>33</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="s">
-        <x:v>38</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="B6" t="s">
-        <x:v>39</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C6" t="s">
-        <x:v>40</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="D6" t="s">
-        <x:v>41</x:v>
+        <x:v>37</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="s">
-        <x:v>42</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B7" t="s">
-        <x:v>43</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C7" t="s">
-        <x:v>44</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="D7" t="s">
-        <x:v>45</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="s">
-        <x:v>46</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="B8" t="s">
-        <x:v>47</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="C8" t="s">
-        <x:v>48</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="D8" t="s">
-        <x:v>49</x:v>
+        <x:v>45</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="s">
-        <x:v>50</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="B9" t="s">
-        <x:v>51</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C9" t="s">
-        <x:v>52</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D9" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="s">
-        <x:v>54</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="B10" t="s">
-        <x:v>55</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="C10" t="s">
-        <x:v>56</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="D10" t="s">
-        <x:v>57</x:v>
+        <x:v>53</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="s">
-        <x:v>58</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="B11" t="s">
-        <x:v>59</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C11" t="s">
-        <x:v>60</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="D11" t="s">
-        <x:v>61</x:v>
+        <x:v>57</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="s">
-        <x:v>62</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="B12" t="s">
-        <x:v>63</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="C12" t="s">
-        <x:v>64</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="D12" t="s">
-        <x:v>65</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="s">
-        <x:v>66</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="B13" t="s">
-        <x:v>67</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C13" t="s">
-        <x:v>68</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="D13" t="s">
-        <x:v>69</x:v>
+        <x:v>65</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="s">
-        <x:v>70</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="B14" t="s">
-        <x:v>71</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C14" t="s">
-        <x:v>72</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="D14" t="s">
-        <x:v>73</x:v>
+        <x:v>69</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="s">
-        <x:v>74</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="B15" t="s">
-        <x:v>75</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="C15" t="s">
-        <x:v>76</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="D15" t="s">
-        <x:v>77</x:v>
+        <x:v>73</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2702,72 +2716,72 @@
   <x:sheetData>
     <x:row r="1" ht="28.049999237060547" customHeight="1">
       <x:c r="A1" s="9" t="s">
-        <x:v>78</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="B1" s="9"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="2" t="s">
-        <x:v>79</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>80</x:v>
+        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="s">
-        <x:v>81</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B3" s="2" t="s">
-        <x:v>82</x:v>
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="2" t="s">
-        <x:v>83</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="B4" s="2" t="s">
-        <x:v>84</x:v>
+        <x:v>80</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="2" t="s">
-        <x:v>85</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="B5" s="2" t="s">
-        <x:v>86</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="2" t="s">
-        <x:v>87</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B6" s="2" t="s">
-        <x:v>88</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="2" t="s">
-        <x:v>89</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="B7" s="2" t="s">
-        <x:v>90</x:v>
+        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="2" t="s">
-        <x:v>91</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="B8" s="2" t="s">
-        <x:v>92</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="2" t="s">
-        <x:v>93</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="B9" s="2" t="s">
-        <x:v>94</x:v>
+        <x:v>90</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Add asset references and music licensing
</commit_message>
<xml_diff>
--- a/asset_manifest.xlsx
+++ b/asset_manifest.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" r:id="R223ae6e09e854af5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset - Trận địa cọc" sheetId="2" r:id="Rd60bef940a1b4ae7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prefix" sheetId="3" r:id="R21c78b134bbe41b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hướng dẫn" sheetId="4" r:id="Rf988d09c8eb84f9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" r:id="R5110a9d3b1ab408f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset - Trận địa cọc" sheetId="2" r:id="Ra207dd75ec4a40c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prefix" sheetId="3" r:id="Rdc25464d1bde4959"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hướng dẫn" sheetId="4" r:id="Rfc9c7ab1c9ba4f5c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -172,9 +172,6 @@
     <x:t xml:space="preserve">Nhạc nền</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">ambient_original.mp3</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">SFX</x:t>
   </x:si>
   <x:si>
@@ -247,15 +244,9 @@
     <x:t xml:space="preserve">2. Đưa lên GitHub</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Giữ nguyên đường dẫn thư mục asset để DEMO hoạt động.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">3. Đường dẫn repo</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Chỉ điền cột Link khi asset đã thực sự được đẩy lên GitHub.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">4. Phần chưa có</x:t>
   </x:si>
   <x:si>
@@ -269,9 +260,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">6. Cách hiểu animation</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Animation dùng tween trong DEMO/game.js, không phải file video dựng sẵn.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">7. Bản quyền</x:t>
@@ -397,7 +385,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="11">
+  <x:cellXfs count="14">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -422,6 +410,15 @@
     <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -696,7 +693,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B9" s="2" t="str">
-        <x:v>Đã bỏ reference khỏi danh sách asset chính; file vẫn giữ trong thư mục REFERENCE.</x:v>
+        <x:v>Đã thêm cột Reference / License cho từng asset; nguồn ngoài chỉ ghi khi có link rõ ràng, asset tự tạo ghi rõ nội bộ.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -704,7 +701,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B10" s="2" t="str">
-        <x:v>Đã bổ sung BGM prototype, trống prototype và script battle call; voice thật còn chờ thu/tạo có cấp phép.</x:v>
+        <x:v>BGM Spirit of Victory đã thay cho hai BGM prototype cũ; dùng chung cho sảnh và gameplay. VO thật vẫn chờ thu/tạo có cấp phép.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -712,7 +709,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B11" s="2" t="str">
-        <x:v>Asset tự tạo và font Be Vietnam Pro có OFL; voice cuối cần xác nhận quyền sử dụng.</x:v>
+        <x:v>Asset tự tạo, font Be Vietnam Pro có OFL; BGM Spirit of Victory dùng theo Pixabay Content License và được ghi nhận là AI-generated.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -753,6 +750,7 @@
     <x:col min="8" max="8" width="32" customWidth="1"/>
     <x:col min="9" max="9" width="55" customWidth="1"/>
     <x:col min="10" max="10" width="12" customWidth="1"/>
+    <x:col min="11" max="11" width="52" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
@@ -786,7 +784,9 @@
       <x:c r="J1" s="1" t="str">
         <x:v>Ưu tiên</x:v>
       </x:c>
-      <x:c r="K1"/>
+      <x:c r="K1" s="11" t="str">
+        <x:v>Reference / License</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="28.950000762939453" customHeight="1">
       <x:c r="A2" s="2" t="n">
@@ -819,7 +819,9 @@
       <x:c r="J2" s="2" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K2"/>
+      <x:c r="K2" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="28.950000762939453" customHeight="1">
       <x:c r="A3" s="2" t="n">
@@ -852,7 +854,9 @@
       <x:c r="J3" s="2" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K3"/>
+      <x:c r="K3" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="28.950000762939453" customHeight="1">
       <x:c r="A4" s="2" t="n">
@@ -885,7 +889,9 @@
       <x:c r="J4" s="2" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K4"/>
+      <x:c r="K4" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="28.950000762939453" customHeight="1">
       <x:c r="A5" s="2" t="n">
@@ -918,7 +924,9 @@
       <x:c r="J5" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K5"/>
+      <x:c r="K5" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="28.950000762939453" customHeight="1">
       <x:c r="A6" s="2" t="n">
@@ -951,7 +959,9 @@
       <x:c r="J6" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K6"/>
+      <x:c r="K6" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="28.950000762939453" customHeight="1">
       <x:c r="A7" s="2" t="n">
@@ -984,7 +994,9 @@
       <x:c r="J7" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K7"/>
+      <x:c r="K7" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="28.950000762939453" customHeight="1">
       <x:c r="A8" s="2" t="n">
@@ -1017,7 +1029,9 @@
       <x:c r="J8" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K8"/>
+      <x:c r="K8" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="28.950000762939453" customHeight="1">
       <x:c r="A9" s="2" t="n">
@@ -1050,7 +1064,9 @@
       <x:c r="J9" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K9"/>
+      <x:c r="K9" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="28.950000762939453" customHeight="1">
       <x:c r="A10" s="2" t="n">
@@ -1083,7 +1099,9 @@
       <x:c r="J10" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K10"/>
+      <x:c r="K10" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="28.950000762939453" customHeight="1">
       <x:c r="A11" s="2" t="n">
@@ -1116,7 +1134,9 @@
       <x:c r="J11" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K11"/>
+      <x:c r="K11" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="28.950000762939453" customHeight="1">
       <x:c r="A12" s="2" t="n">
@@ -1149,7 +1169,9 @@
       <x:c r="J12" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K12"/>
+      <x:c r="K12" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="28.950000762939453" customHeight="1">
       <x:c r="A13" s="2" t="n">
@@ -1182,7 +1204,9 @@
       <x:c r="J13" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K13"/>
+      <x:c r="K13" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="28.950000762939453" customHeight="1">
       <x:c r="A14" s="2" t="n">
@@ -1215,7 +1239,9 @@
       <x:c r="J14" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K14"/>
+      <x:c r="K14" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="28.950000762939453" customHeight="1">
       <x:c r="A15" s="2" t="n">
@@ -1248,7 +1274,9 @@
       <x:c r="J15" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K15"/>
+      <x:c r="K15" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="28.950000762939453" customHeight="1">
       <x:c r="A16" s="2" t="n">
@@ -1281,7 +1309,9 @@
       <x:c r="J16" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K16"/>
+      <x:c r="K16" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="28.950000762939453" customHeight="1">
       <x:c r="A17" s="2" t="n">
@@ -1294,10 +1324,10 @@
         <x:v>BGM</x:v>
       </x:c>
       <x:c r="D17" s="2" t="str">
-        <x:v>lobby_theme</x:v>
+        <x:v>BGM_SpiritOfVictory_Pixabay</x:v>
       </x:c>
       <x:c r="E17" s="2" t="str">
-        <x:v>Nhạc nền sảnh prototype loop 16 giây, tự tạo; bản chính thức có thể remaster thành 60–90 giây</x:v>
+        <x:v>Nhạc nền sảnh, phát loop 1 file dùng chung</x:v>
       </x:c>
       <x:c r="F17" s="2" t="str">
         <x:v>1</x:v>
@@ -1306,15 +1336,17 @@
         <x:v>Đã có</x:v>
       </x:c>
       <x:c r="H17" s="2" t="str">
-        <x:v>https://github.com/mil352k5-ux/MiniGame_TranDiaCocBD/blob/main/BGM/lobby_theme_prototype.wav</x:v>
+        <x:v>https://github.com/mil352k5-ux/MiniGame_TranDiaCocBD/blob/main/BGM/spirit_of_victory_pixabay.mp3</x:v>
       </x:c>
       <x:c r="I17" s="2" t="str">
-        <x:v>BGM/lobby_theme_prototype.wav</x:v>
+        <x:v>BGM/spirit_of_victory_pixabay.mp3</x:v>
       </x:c>
       <x:c r="J17" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K17"/>
+      <x:c r="K17" s="13" t="str">
+        <x:v>Pixabay – Spirit of Victory (AI-generated): https://pixabay.com/music/main-title-spirit-of-victory-331312/</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="28.950000762939453" customHeight="1">
       <x:c r="A18" s="2" t="n">
@@ -1347,7 +1379,9 @@
       <x:c r="J18" s="2" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K18"/>
+      <x:c r="K18" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="28.950000762939453" customHeight="1">
       <x:c r="A19" s="2" t="n">
@@ -1380,7 +1414,9 @@
       <x:c r="J19" s="2" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K19"/>
+      <x:c r="K19" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="28.950000762939453" customHeight="1">
       <x:c r="A20" s="2" t="n">
@@ -1413,7 +1449,9 @@
       <x:c r="J20" s="2" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K20"/>
+      <x:c r="K20" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="28.950000762939453" customHeight="1">
       <x:c r="A21" s="2" t="n">
@@ -1446,7 +1484,9 @@
       <x:c r="J21" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K21"/>
+      <x:c r="K21" s="13" t="str">
+        <x:v>AI-generated trong cuộc hội thoại; chỉ là minh họa, không phải tư liệu lịch sử</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="28.950000762939453" customHeight="1">
       <x:c r="A22" s="2" t="n">
@@ -1479,7 +1519,9 @@
       <x:c r="J22" s="2" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K22"/>
+      <x:c r="K22" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="28.950000762939453" customHeight="1">
       <x:c r="A23" s="2" t="n">
@@ -1512,7 +1554,9 @@
       <x:c r="J23" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K23"/>
+      <x:c r="K23" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="28.950000762939453" customHeight="1">
       <x:c r="A24" s="2" t="n">
@@ -1545,7 +1589,9 @@
       <x:c r="J24" s="2" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K24"/>
+      <x:c r="K24" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="28.950000762939453" customHeight="1">
       <x:c r="A25" s="2" t="n">
@@ -1578,7 +1624,9 @@
       <x:c r="J25" s="2" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K25"/>
+      <x:c r="K25" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="28.950000762939453" customHeight="1">
       <x:c r="A26" s="2" t="n">
@@ -1611,7 +1659,9 @@
       <x:c r="J26" s="2" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K26"/>
+      <x:c r="K26" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="28.950000762939453" customHeight="1">
       <x:c r="A27" s="2" t="n">
@@ -1644,7 +1694,9 @@
       <x:c r="J27" s="2" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="K27"/>
+      <x:c r="K27" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="28.950000762939453" customHeight="1">
       <x:c r="A28" s="2" t="n">
@@ -1657,10 +1709,10 @@
         <x:v>BGM</x:v>
       </x:c>
       <x:c r="D28" s="2" t="str">
-        <x:v>gameplay_theme</x:v>
+        <x:v>BGM_SpiritOfVictory_Pixabay</x:v>
       </x:c>
       <x:c r="E28" s="2" t="str">
-        <x:v>Nhạc nền gameplay prototype loop 16 giây, tự tạo; bản chính thức có thể mở rộng 90–120 giây</x:v>
+        <x:v>Nhạc nền gameplay, phát loop 1 file dùng chung</x:v>
       </x:c>
       <x:c r="F28" s="2" t="str">
         <x:v>1</x:v>
@@ -1669,15 +1721,17 @@
         <x:v>Đã có</x:v>
       </x:c>
       <x:c r="H28" s="2" t="str">
-        <x:v>https://github.com/mil352k5-ux/MiniGame_TranDiaCocBD/blob/main/BGM/gameplay_theme_prototype.wav</x:v>
+        <x:v>https://github.com/mil352k5-ux/MiniGame_TranDiaCocBD/blob/main/BGM/spirit_of_victory_pixabay.mp3</x:v>
       </x:c>
       <x:c r="I28" s="2" t="str">
-        <x:v>BGM/gameplay_theme_prototype.wav</x:v>
+        <x:v>BGM/spirit_of_victory_pixabay.mp3</x:v>
       </x:c>
       <x:c r="J28" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K28"/>
+      <x:c r="K28" s="13" t="str">
+        <x:v>Pixabay – Spirit of Victory (AI-generated): https://pixabay.com/music/main-title-spirit-of-victory-331312/</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="28.950000762939453" customHeight="1">
       <x:c r="A29" s="2" t="n">
@@ -1710,7 +1764,9 @@
       <x:c r="J29" s="2" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K29"/>
+      <x:c r="K29" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="28.950000762939453" customHeight="1">
       <x:c r="A30" s="2" t="n">
@@ -1743,7 +1799,9 @@
       <x:c r="J30" s="2" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K30"/>
+      <x:c r="K30" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="28.950000762939453" customHeight="1">
       <x:c r="A31" s="2" t="n">
@@ -1776,7 +1834,9 @@
       <x:c r="J31" s="2" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K31"/>
+      <x:c r="K31" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="28.950000762939453" customHeight="1">
       <x:c r="A32" s="2" t="n">
@@ -1809,7 +1869,9 @@
       <x:c r="J32" s="2" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K32"/>
+      <x:c r="K32" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="28.950000762939453" customHeight="1">
       <x:c r="A33" s="2" t="n">
@@ -1842,7 +1904,9 @@
       <x:c r="J33" s="2" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K33"/>
+      <x:c r="K33" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="28.950000762939453" customHeight="1">
       <x:c r="A34" s="2" t="n">
@@ -1875,7 +1939,9 @@
       <x:c r="J34" s="2" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="K34"/>
+      <x:c r="K34" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="28.950000762939453" customHeight="1">
       <x:c r="A35" s="2" t="n">
@@ -1908,7 +1974,9 @@
       <x:c r="J35" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K35"/>
+      <x:c r="K35" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="28.950000762939453" customHeight="1">
       <x:c r="A36" s="2" t="n">
@@ -1941,7 +2009,9 @@
       <x:c r="J36" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K36"/>
+      <x:c r="K36" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="28.950000762939453" customHeight="1">
       <x:c r="A37" s="2" t="n">
@@ -1974,7 +2044,9 @@
       <x:c r="J37" s="2" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K37"/>
+      <x:c r="K37" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="28.950000762939453" customHeight="1">
       <x:c r="A38" s="2" t="n">
@@ -2007,7 +2079,9 @@
       <x:c r="J38" s="2" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K38"/>
+      <x:c r="K38" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="28.950000762939453" customHeight="1">
       <x:c r="A39" s="2" t="n">
@@ -2040,7 +2114,9 @@
       <x:c r="J39" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K39"/>
+      <x:c r="K39" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="28.950000762939453" customHeight="1">
       <x:c r="A40" s="2" t="n">
@@ -2073,7 +2149,9 @@
       <x:c r="J40" s="2" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K40"/>
+      <x:c r="K40" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="28.950000762939453" customHeight="1">
       <x:c r="A41" s="2" t="n">
@@ -2106,7 +2184,9 @@
       <x:c r="J41" s="2" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K41"/>
+      <x:c r="K41" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="28.950000762939453" customHeight="1">
       <x:c r="A42" s="2" t="n">
@@ -2139,7 +2219,9 @@
       <x:c r="J42" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K42"/>
+      <x:c r="K42" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="28.950000762939453" customHeight="1">
       <x:c r="A43" s="2" t="n">
@@ -2172,7 +2254,9 @@
       <x:c r="J43" s="2" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="K43"/>
+      <x:c r="K43" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="28.950000762939453" customHeight="1">
       <x:c r="A44" s="2" t="n">
@@ -2205,7 +2289,9 @@
       <x:c r="J44" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K44"/>
+      <x:c r="K44" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="28.950000762939453" customHeight="1">
       <x:c r="A45" s="2" t="n">
@@ -2238,7 +2324,9 @@
       <x:c r="J45" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K45"/>
+      <x:c r="K45" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="28.950000762939453" customHeight="1">
       <x:c r="A46" s="2" t="n">
@@ -2271,7 +2359,9 @@
       <x:c r="J46" s="2" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K46"/>
+      <x:c r="K46" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="28.950000762939453" customHeight="1">
       <x:c r="A47" s="2" t="n">
@@ -2304,7 +2394,9 @@
       <x:c r="J47" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K47"/>
+      <x:c r="K47" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="28.950000762939453" customHeight="1">
       <x:c r="A48" s="2" t="n">
@@ -2337,7 +2429,9 @@
       <x:c r="J48" s="2" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K48"/>
+      <x:c r="K48" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" t="n">
@@ -2370,7 +2464,9 @@
       <x:c r="J49" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K49"/>
+      <x:c r="K49" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" t="n">
@@ -2386,13 +2482,13 @@
         <x:v>ambient_original</x:v>
       </x:c>
       <x:c r="E50" t="str">
-        <x:v>Nhạc nền tổng hợp đơn giản, lặp 20 giây</x:v>
+        <x:v>Nhạc nền prototype cũ; giữ để tham khảo, không dùng trong demo hiện tại</x:v>
       </x:c>
       <x:c r="F50" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G50" t="str">
-        <x:v>Đã có</x:v>
+        <x:v>Bản nháp – không dùng</x:v>
       </x:c>
       <x:c r="H50" t="str">
         <x:v>https://github.com/mil352k5-ux/MiniGame_TranDiaCocBD/blob/main/BGM/ambient_original.mp3</x:v>
@@ -2403,7 +2499,9 @@
       <x:c r="J50" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K50"/>
+      <x:c r="K50" s="13" t="str">
+        <x:v>Nội bộ / code-synthesized; bản nháp, không dùng trong demo hiện tại</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" t="n">
@@ -2436,7 +2534,9 @@
       <x:c r="J51" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K51"/>
+      <x:c r="K51" s="13" t="str">
+        <x:v>Google Fonts – Be Vietnam Pro: https://fonts.google.com/specimen/Be+Vietnam+Pro</x:v>
+      </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" t="n">
@@ -2469,7 +2569,9 @@
       <x:c r="J52" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K52"/>
+      <x:c r="K52" s="13" t="str">
+        <x:v>Nội bộ / tự tạo trong dự án</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -2627,78 +2729,78 @@
       <x:c r="C10" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="D10" t="s">
-        <x:v>53</x:v>
+      <x:c r="D10" t="str">
+        <x:v>spirit_of_victory_pixabay.mp3</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="B11" t="s">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="B11" t="s">
+      <x:c r="C11" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="C11" t="s">
+      <x:c r="D11" t="s">
         <x:v>56</x:v>
-      </x:c>
-      <x:c r="D11" t="s">
-        <x:v>57</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B12" t="s">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="B12" t="s">
+      <x:c r="C12" t="s">
         <x:v>59</x:v>
       </x:c>
-      <x:c r="C12" t="s">
+      <x:c r="D12" t="s">
         <x:v>60</x:v>
-      </x:c>
-      <x:c r="D12" t="s">
-        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="B13" t="s">
         <x:v>62</x:v>
       </x:c>
-      <x:c r="B13" t="s">
+      <x:c r="C13" t="s">
         <x:v>63</x:v>
       </x:c>
-      <x:c r="C13" t="s">
+      <x:c r="D13" t="s">
         <x:v>64</x:v>
-      </x:c>
-      <x:c r="D13" t="s">
-        <x:v>65</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="s">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="B14" t="s">
         <x:v>66</x:v>
       </x:c>
-      <x:c r="B14" t="s">
+      <x:c r="C14" t="s">
         <x:v>67</x:v>
       </x:c>
-      <x:c r="C14" t="s">
+      <x:c r="D14" t="s">
         <x:v>68</x:v>
-      </x:c>
-      <x:c r="D14" t="s">
-        <x:v>69</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="B15" t="s">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="B15" t="s">
+      <x:c r="C15" t="s">
         <x:v>71</x:v>
       </x:c>
-      <x:c r="C15" t="s">
+      <x:c r="D15" t="s">
         <x:v>72</x:v>
-      </x:c>
-      <x:c r="D15" t="s">
-        <x:v>73</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2716,72 +2818,72 @@
   <x:sheetData>
     <x:row r="1" ht="28.049999237060547" customHeight="1">
       <x:c r="A1" s="9" t="s">
-        <x:v>74</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="B1" s="9"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="2" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="B2" s="2" t="s">
         <x:v>75</x:v>
-      </x:c>
-      <x:c r="B2" s="2" t="s">
-        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="s">
-        <x:v>77</x:v>
-      </x:c>
-      <x:c r="B3" s="2" t="s">
-        <x:v>78</x:v>
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="str">
+        <x:v>Giữ nguyên đường dẫn thư mục asset để DEMO hoạt động. Cột Link là file trong GitHub; cột Reference / License là nguồn hoặc giấy phép.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="2" t="s">
-        <x:v>79</x:v>
-      </x:c>
-      <x:c r="B4" s="2" t="s">
-        <x:v>80</x:v>
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="B4" s="2" t="str">
+        <x:v>Phần chưa có: không đánh dấu hoàn thành những asset hi-res/VO/font chưa được tạo; chỉ điền reference khi có nguồn xác minh được.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="2" t="s">
-        <x:v>81</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="B5" s="2" t="s">
-        <x:v>82</x:v>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="2" t="s">
-        <x:v>83</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="B6" s="2" t="s">
-        <x:v>84</x:v>
+        <x:v>81</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="2" t="s">
-        <x:v>85</x:v>
-      </x:c>
-      <x:c r="B7" s="2" t="s">
-        <x:v>86</x:v>
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="B7" s="2" t="str">
+        <x:v>Bản quyền: kiểm tra cột Reference / License trước khi bàn giao; không sử dụng hình và âm thanh từ Knife Hit hay game khác.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="2" t="s">
-        <x:v>87</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B8" s="2" t="s">
-        <x:v>88</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="2" t="s">
-        <x:v>89</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="B9" s="2" t="s">
-        <x:v>90</x:v>
+        <x:v>86</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>